<commit_message>
Proximity in morning mode
</commit_message>
<xml_diff>
--- a/bus_details.xlsx
+++ b/bus_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pruthivi\OneDrive\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pruthivi\comb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C5F1F6-2992-4E8C-9609-F9FB36618D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29042EB7-9115-4A6F-8482-E59A0FA1397E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8460AF98-2045-4371-B0FF-AB609739834E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8460AF98-2045-4371-B0FF-AB609739834E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t>bus_no</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>meppur</t>
+  </si>
+  <si>
+    <t>kumananchavadi</t>
   </si>
 </sst>
 </file>
@@ -533,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DB043-1D73-498E-9279-AF026CDE3BBE}">
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="76" customWidth="1"/>
@@ -1059,6 +1062,14 @@
         <v>41</v>
       </c>
     </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>1</v>
+      </c>
+      <c r="B66" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>